<commit_message>
Fix white font on summary rows in sort_inventory and parse_manifest
First row of each variant block gets bold black font on cols A-E (visible).
Subsequent rows stay white (hidden repeated labels).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventory_master.xlsx
+++ b/inventory_master.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,12 @@
     <font>
       <name val="Arial"/>
       <color rgb="FFFF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -356,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -541,6 +547,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1062,27 +1080,27 @@
       <c r="L2" s="24" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="66" t="inlineStr">
+      <c r="A3" s="70" t="inlineStr">
         <is>
           <t>Altea Double Door</t>
         </is>
       </c>
-      <c r="B3" s="67" t="inlineStr">
+      <c r="B3" s="71" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C3" s="67" t="inlineStr">
+      <c r="C3" s="71" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D3" s="67" t="inlineStr">
+      <c r="D3" s="71" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E3" s="67" t="inlineStr">
+      <c r="E3" s="71" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1294,27 +1312,27 @@
       <c r="L8" s="39" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="34" t="inlineStr">
+      <c r="A9" s="72" t="inlineStr">
         <is>
           <t>Altea Double Door</t>
         </is>
       </c>
-      <c r="B9" s="35" t="inlineStr">
+      <c r="B9" s="73" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C9" s="35" t="inlineStr">
+      <c r="C9" s="73" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D9" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E9" s="35" t="inlineStr">
+      <c r="D9" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E9" s="73" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -1602,27 +1620,27 @@
       <c r="L16" s="39" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="34" t="inlineStr">
+      <c r="A17" s="72" t="inlineStr">
         <is>
           <t>Altea Double Door</t>
         </is>
       </c>
-      <c r="B17" s="35" t="inlineStr">
+      <c r="B17" s="73" t="inlineStr">
         <is>
           <t>36" x 96"</t>
         </is>
       </c>
-      <c r="C17" s="35" t="inlineStr">
+      <c r="C17" s="73" t="inlineStr">
         <is>
           <t>Oil-Rubbed Bronze</t>
         </is>
       </c>
-      <c r="D17" s="35" t="inlineStr">
+      <c r="D17" s="73" t="inlineStr">
         <is>
           <t>Right Outswing</t>
         </is>
       </c>
-      <c r="E17" s="35" t="inlineStr">
+      <c r="E17" s="73" t="inlineStr">
         <is>
           <t>Sidelite</t>
         </is>
@@ -1666,27 +1684,27 @@
       <c r="L18" s="39" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="72" t="inlineStr">
         <is>
           <t>Altea Double Door</t>
         </is>
       </c>
-      <c r="B19" s="35" t="inlineStr">
+      <c r="B19" s="73" t="inlineStr">
         <is>
           <t>72" x 80"</t>
         </is>
       </c>
-      <c r="C19" s="35" t="inlineStr">
+      <c r="C19" s="73" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D19" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E19" s="35" t="inlineStr">
+      <c r="D19" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E19" s="73" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1870,27 +1888,27 @@
       <c r="L24" s="42" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="66" t="inlineStr">
+      <c r="A25" s="70" t="inlineStr">
         <is>
           <t>Cordova Sliding Window</t>
         </is>
       </c>
-      <c r="B25" s="67" t="inlineStr">
+      <c r="B25" s="71" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C25" s="67" t="inlineStr">
+      <c r="C25" s="71" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D25" s="67" t="inlineStr">
+      <c r="D25" s="71" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E25" s="67" t="inlineStr">
+      <c r="E25" s="71" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -2144,27 +2162,27 @@
       <c r="L31" s="39" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="34" t="inlineStr">
+      <c r="A32" s="72" t="inlineStr">
         <is>
           <t>Cordova Sliding Window</t>
         </is>
       </c>
-      <c r="B32" s="35" t="inlineStr">
+      <c r="B32" s="73" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C32" s="35" t="inlineStr">
+      <c r="C32" s="73" t="inlineStr">
         <is>
           <t>Oil-Rubbed Bronze</t>
         </is>
       </c>
-      <c r="D32" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E32" s="35" t="inlineStr">
+      <c r="D32" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E32" s="73" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2292,27 +2310,27 @@
       <c r="L35" s="39" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="34" t="inlineStr">
+      <c r="A36" s="72" t="inlineStr">
         <is>
           <t>Cordova Sliding Window</t>
         </is>
       </c>
-      <c r="B36" s="35" t="inlineStr">
+      <c r="B36" s="73" t="inlineStr">
         <is>
           <t>36" x 96"</t>
         </is>
       </c>
-      <c r="C36" s="35" t="inlineStr">
+      <c r="C36" s="73" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D36" s="35" t="inlineStr">
+      <c r="D36" s="73" t="inlineStr">
         <is>
           <t>Right Outswing</t>
         </is>
       </c>
-      <c r="E36" s="35" t="inlineStr">
+      <c r="E36" s="73" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -2356,27 +2374,27 @@
       <c r="L37" s="39" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="34" t="inlineStr">
+      <c r="A38" s="72" t="inlineStr">
         <is>
           <t>Cordova Sliding Window</t>
         </is>
       </c>
-      <c r="B38" s="35" t="inlineStr">
+      <c r="B38" s="73" t="inlineStr">
         <is>
           <t>48" x 36"</t>
         </is>
       </c>
-      <c r="C38" s="35" t="inlineStr">
+      <c r="C38" s="73" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D38" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E38" s="35" t="inlineStr">
+      <c r="D38" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E38" s="73" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2896,27 +2914,27 @@
       <c r="L51" s="42" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="66" t="inlineStr">
+      <c r="A52" s="70" t="inlineStr">
         <is>
           <t>Granada Bi-fold Door</t>
         </is>
       </c>
-      <c r="B52" s="67" t="inlineStr">
+      <c r="B52" s="71" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C52" s="67" t="inlineStr">
+      <c r="C52" s="71" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D52" s="67" t="inlineStr">
+      <c r="D52" s="71" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E52" s="67" t="inlineStr">
+      <c r="E52" s="71" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -3254,27 +3272,27 @@
       <c r="L60" s="39" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="34" t="inlineStr">
+      <c r="A61" s="72" t="inlineStr">
         <is>
           <t>Granada Bi-fold Door</t>
         </is>
       </c>
-      <c r="B61" s="35" t="inlineStr">
+      <c r="B61" s="73" t="inlineStr">
         <is>
           <t>36" x 96"</t>
         </is>
       </c>
-      <c r="C61" s="35" t="inlineStr">
+      <c r="C61" s="73" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D61" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E61" s="35" t="inlineStr">
+      <c r="D61" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E61" s="73" t="inlineStr">
         <is>
           <t>Sidelite</t>
         </is>
@@ -3360,27 +3378,27 @@
       <c r="L63" s="39" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="34" t="inlineStr">
+      <c r="A64" s="72" t="inlineStr">
         <is>
           <t>Granada Bi-fold Door</t>
         </is>
       </c>
-      <c r="B64" s="35" t="inlineStr">
+      <c r="B64" s="73" t="inlineStr">
         <is>
           <t>96" x 80"</t>
         </is>
       </c>
-      <c r="C64" s="35" t="inlineStr">
+      <c r="C64" s="73" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D64" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E64" s="35" t="inlineStr">
+      <c r="D64" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E64" s="73" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -3522,27 +3540,27 @@
       <c r="L68" s="42" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="66" t="inlineStr">
+      <c r="A69" s="70" t="inlineStr">
         <is>
           <t>Malaga Single Door</t>
         </is>
       </c>
-      <c r="B69" s="67" t="inlineStr">
+      <c r="B69" s="71" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C69" s="67" t="inlineStr">
+      <c r="C69" s="71" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D69" s="67" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E69" s="67" t="inlineStr">
+      <c r="D69" s="71" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E69" s="71" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -3712,27 +3730,27 @@
       <c r="L73" s="39" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="34" t="inlineStr">
+      <c r="A74" s="72" t="inlineStr">
         <is>
           <t>Malaga Single Door</t>
         </is>
       </c>
-      <c r="B74" s="35" t="inlineStr">
+      <c r="B74" s="73" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C74" s="35" t="inlineStr">
+      <c r="C74" s="73" t="inlineStr">
         <is>
           <t>Gunmetal</t>
         </is>
       </c>
-      <c r="D74" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E74" s="35" t="inlineStr">
+      <c r="D74" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E74" s="73" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -4378,27 +4396,27 @@
       <c r="L90" s="42" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="66" t="inlineStr">
+      <c r="A91" s="70" t="inlineStr">
         <is>
           <t>Sevilla French Door</t>
         </is>
       </c>
-      <c r="B91" s="67" t="inlineStr">
+      <c r="B91" s="71" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C91" s="67" t="inlineStr">
+      <c r="C91" s="71" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D91" s="67" t="inlineStr">
+      <c r="D91" s="71" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E91" s="67" t="inlineStr">
+      <c r="E91" s="71" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -4610,27 +4628,27 @@
       <c r="L96" s="39" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="34" t="inlineStr">
+      <c r="A97" s="72" t="inlineStr">
         <is>
           <t>Sevilla French Door</t>
         </is>
       </c>
-      <c r="B97" s="35" t="inlineStr">
+      <c r="B97" s="73" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C97" s="35" t="inlineStr">
+      <c r="C97" s="73" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D97" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E97" s="35" t="inlineStr">
+      <c r="D97" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E97" s="73" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -4918,27 +4936,27 @@
       <c r="L104" s="39" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="34" t="inlineStr">
+      <c r="A105" s="72" t="inlineStr">
         <is>
           <t>Sevilla French Door</t>
         </is>
       </c>
-      <c r="B105" s="35" t="inlineStr">
+      <c r="B105" s="73" t="inlineStr">
         <is>
           <t>72" x 80"</t>
         </is>
       </c>
-      <c r="C105" s="35" t="inlineStr">
+      <c r="C105" s="73" t="inlineStr">
         <is>
           <t>Matte White</t>
         </is>
       </c>
-      <c r="D105" s="35" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E105" s="35" t="inlineStr">
+      <c r="D105" s="73" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E105" s="73" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -5164,27 +5182,27 @@
       <c r="L111" s="42" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="66" t="inlineStr">
+      <c r="A112" s="70" t="inlineStr">
         <is>
           <t>Valencia Single Door</t>
         </is>
       </c>
-      <c r="B112" s="67" t="inlineStr">
+      <c r="B112" s="71" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C112" s="67" t="inlineStr">
+      <c r="C112" s="71" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D112" s="67" t="inlineStr">
-        <is>
-          <t>Left Inswing</t>
-        </is>
-      </c>
-      <c r="E112" s="67" t="inlineStr">
+      <c r="D112" s="71" t="inlineStr">
+        <is>
+          <t>Left Inswing</t>
+        </is>
+      </c>
+      <c r="E112" s="71" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -5594,27 +5612,27 @@
       <c r="L122" s="39" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="34" t="inlineStr">
+      <c r="A123" s="72" t="inlineStr">
         <is>
           <t>Valencia Single Door</t>
         </is>
       </c>
-      <c r="B123" s="35" t="inlineStr">
+      <c r="B123" s="73" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C123" s="35" t="inlineStr">
+      <c r="C123" s="73" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D123" s="35" t="inlineStr">
+      <c r="D123" s="73" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E123" s="35" t="inlineStr">
+      <c r="E123" s="73" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -5910,27 +5928,27 @@
       <c r="L130" s="39" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="34" t="inlineStr">
+      <c r="A131" s="72" t="inlineStr">
         <is>
           <t>Valencia Single Door</t>
         </is>
       </c>
-      <c r="B131" s="35" t="inlineStr">
+      <c r="B131" s="73" t="inlineStr">
         <is>
           <t>36" x 96"</t>
         </is>
       </c>
-      <c r="C131" s="35" t="inlineStr">
+      <c r="C131" s="73" t="inlineStr">
         <is>
           <t>Oil-Rubbed Bronze</t>
         </is>
       </c>
-      <c r="D131" s="35" t="inlineStr">
+      <c r="D131" s="73" t="inlineStr">
         <is>
           <t>Right Outswing</t>
         </is>
       </c>
-      <c r="E131" s="35" t="inlineStr">
+      <c r="E131" s="73" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>

</xml_diff>